<commit_message>
Đã cập nhật lại, làm sạch code (tách file và đổi tên file) cho dễ quản lý, mọi ng có thể cài ứng dụng được
</commit_message>
<xml_diff>
--- a/data/users_data.xlsx
+++ b/data/users_data.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="13476" windowHeight="7392" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -412,11 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="19.6640625" customWidth="1" min="7" max="7"/>
-  </cols>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -501,20 +499,14 @@
           <t>phat@gmail.com</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1234567</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>36633663</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="C2" t="n">
+        <v>1234567</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36633663</v>
+      </c>
+      <c r="E2" t="n">
+        <v>18</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -524,12 +516,55 @@
           <t>2026-03-27</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
         <v>0.360759158929189</v>
       </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
-        <v>61.38298732042313</v>
-      </c>
+        <v>61.82553251187007</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kiet</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kietlattt@gmail.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>36632</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>